<commit_message>
used: finish OM bot
</commit_message>
<xml_diff>
--- a/98 - Excels/Open-OMs.xlsx
+++ b/98 - Excels/Open-OMs.xlsx
@@ -1,63 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\feb3ct\Desktop\PyAutomateSAP\98 - Excels\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88980A8F-6AD4-484C-8CBC-0602AF1FBC5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="3">
-  <si>
-    <t>OM</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Encerrado!</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -65,44 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -390,155 +408,284 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>OM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>5206488</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
         <v>5206409</v>
       </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
         <v>5204338</v>
       </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
         <v>5205664</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>5205623</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
         <v>5205946</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>5204785</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
         <v>5206055</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
         <v>5206317</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>5205946</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
         <v>5204389</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
         <v>685601436680</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
         <v>685601438071</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
         <v>685601417176</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ordem pendente!</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
         <v>685601426608</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
         <v>685601417177</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
         <v>685601414700</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
         <v>685601429585</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
         <v>685601425282</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
         <v>685601427688</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
         <v>685601418035</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
         <v>685601420292</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
         <v>685601421139</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
         <v>685601429632</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
         <v>685601424427</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
         <v>685601434381</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: finish om upd
</commit_message>
<xml_diff>
--- a/98 - Excels/Open-OMs.xlsx
+++ b/98 - Excels/Open-OMs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\98 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4DFB7F-ADE4-4354-AE89-F1A12E7E49D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0602AC-1273-4E9A-80EC-3D901E9FD42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="290">
   <si>
     <t>OM</t>
   </si>
@@ -887,6 +887,9 @@
   </si>
   <si>
     <t>5210614</t>
+  </si>
+  <si>
+    <t>Encerrado</t>
   </si>
 </sst>
 </file>
@@ -1245,553 +1248,844 @@
       <c r="A2" t="s">
         <v>34</v>
       </c>
+      <c r="B2" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>35</v>
       </c>
+      <c r="B3" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>36</v>
       </c>
+      <c r="B4" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>37</v>
       </c>
+      <c r="B5" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>38</v>
       </c>
+      <c r="B6" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>39</v>
       </c>
+      <c r="B7" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>40</v>
       </c>
+      <c r="B8" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>41</v>
       </c>
+      <c r="B9" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>42</v>
       </c>
+      <c r="B10" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
+      <c r="B11" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>43</v>
       </c>
+      <c r="B12" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>44</v>
       </c>
+      <c r="B13" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
+      <c r="B14" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>46</v>
       </c>
+      <c r="B15" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B70" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B71" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B72" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B73" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B78" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B82" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B87" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B89" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B91" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B92" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B93" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B94" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B95" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B96" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B97" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B98" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>142</v>
       </c>

</xml_diff>